<commit_message>
Correción en uno de los archivos de prueba
</commit_message>
<xml_diff>
--- a/backend/test-files/Facturas-prueba1.xlsx
+++ b/backend/test-files/Facturas-prueba1.xlsx
@@ -1,37 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30219"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DEE44640-FC4B-4E7A-B4CE-CE3E0185EA6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView/>
   </bookViews>
   <sheets>
-    <sheet name="Receivable Invoice Detail" sheetId="1" r:id="rId1"/>
+    <sheet r:id="rId1" name="Receivable Invoice Detail" sheetId="1"/>
   </sheets>
-  <calcPr calcId="191028"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0" iterateCount="100" iterateDelta="0.001"/>
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>Receivable Invoice Detail</t>
   </si>
@@ -126,47 +130,58 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="dd\ mmm\ yyyy"/>
-    <numFmt numFmtId="165" formatCode="#,##0.0000;\(#,##0.0000\)"/>
-    <numFmt numFmtId="166" formatCode="#,##0.00;\(#,##0.00\)"/>
+    <numFmt numFmtId="406" formatCode="dd\ mmm\ yyyy"/>
+    <numFmt numFmtId="407" formatCode="#,##0.0000;\(#,##0.0000\)"/>
+    <numFmt numFmtId="408" formatCode="#,##0.00;\(#,##0.00\)"/>
   </numFmts>
   <fonts count="7">
     <font>
+      <b val="0"/>
+      <i val="0"/>
       <sz val="9"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
+      <b val="0"/>
+      <i val="0"/>
       <sz val="14"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <i val="0"/>
       <sz val="14"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
+      <b val="0"/>
+      <i val="0"/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
+      <b val="0"/>
+      <i val="0"/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <i val="0"/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <i val="0"/>
       <sz val="9"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -207,71 +222,86 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="406" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="407" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="408" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="407" fontId="0" fillId="0" borderId="2" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="408" fontId="0" fillId="0" borderId="2" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="407" fontId="6" fillId="0" borderId="2" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
+    <cellStyle name="Normal" xfId="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+  <bag type="DXFComplements" extRef="DXFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -317,7 +347,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -369,7 +399,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -430,166 +460,190 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{5864CF8A-B883-4098-AE8F-0AF5F398E561}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:M46"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultRowHeight="12.75" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="85.7109375" customWidth="1"/>
-    <col min="2" max="2" width="23.28515625" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" customWidth="1"/>
-    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="2" max="2" width="23.28125" customWidth="1"/>
+    <col min="3" max="3" width="14.28125" customWidth="1"/>
+    <col min="4" max="4" width="22.00390625" customWidth="1"/>
     <col min="5" max="5" width="11.7109375" customWidth="1"/>
-    <col min="6" max="6" width="12.28515625" customWidth="1"/>
-    <col min="7" max="7" width="100" customWidth="1"/>
+    <col min="6" max="6" width="12.28125" customWidth="1"/>
+    <col min="7" max="7" width="100.00390625" customWidth="1"/>
     <col min="8" max="8" width="10.7109375" customWidth="1"/>
-    <col min="9" max="9" width="25.85546875" customWidth="1"/>
-    <col min="10" max="10" width="24.42578125" customWidth="1"/>
-    <col min="11" max="11" width="14.85546875" customWidth="1"/>
-    <col min="12" max="12" width="16.85546875" customWidth="1"/>
+    <col min="9" max="9" width="25.8515625" customWidth="1"/>
+    <col min="10" max="10" width="24.421875" customWidth="1"/>
+    <col min="11" max="11" width="14.8515625" customWidth="1"/>
+    <col min="12" max="12" width="16.8515625" customWidth="1"/>
     <col min="13" max="13" width="10.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="1" customFormat="1" ht="16.7" customHeight="1">
+    <row r="1" ht="16.5" customHeight="1" s="1" customFormat="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -606,7 +660,7 @@
       <c r="L1" s="2"/>
       <c r="M1" s="2"/>
     </row>
-    <row r="2" spans="1:13" s="3" customFormat="1" ht="14.45" customHeight="1">
+    <row r="2" ht="14.25" customHeight="1" s="3" customFormat="1">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -623,7 +677,7 @@
       <c r="L2" s="4"/>
       <c r="M2" s="4"/>
     </row>
-    <row r="3" spans="1:13" s="3" customFormat="1" ht="14.45" customHeight="1">
+    <row r="3" ht="14.25" customHeight="1" s="3" customFormat="1">
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
@@ -640,14 +694,14 @@
       <c r="L3" s="4"/>
       <c r="M3" s="4"/>
     </row>
-    <row r="4" spans="1:13" ht="13.35" customHeight="1"/>
-    <row r="5" spans="1:13" ht="10.9" customHeight="1">
+    <row r="4" ht="13.5" customHeight="1"/>
+    <row r="5" ht="11.25" customHeight="1">
       <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="13.35" customHeight="1"/>
-    <row r="7" spans="1:13" s="6" customFormat="1" ht="12.2" customHeight="1">
+    <row r="6" ht="13.5" customHeight="1"/>
+    <row r="7" ht="12" customHeight="1" s="6" customFormat="1">
       <c r="A7" s="7" t="s">
         <v>4</v>
       </c>
@@ -688,7 +742,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="10.9" customHeight="1">
+    <row r="8" ht="11.25" customHeight="1">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -701,7 +755,9 @@
       <c r="D8" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="9"/>
+      <c r="E8" s="9">
+        <v>59863</v>
+      </c>
       <c r="F8" s="9" t="s">
         <v>20</v>
       </c>
@@ -727,7 +783,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="10.9" customHeight="1">
+    <row r="9" ht="11.25" customHeight="1">
       <c r="A9" s="9" t="s">
         <v>17</v>
       </c>
@@ -740,7 +796,9 @@
       <c r="D9" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E9" s="13"/>
+      <c r="E9" s="13">
+        <v>59863</v>
+      </c>
       <c r="F9" s="13" t="s">
         <v>20</v>
       </c>
@@ -766,7 +824,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="10.9" customHeight="1">
+    <row r="10" ht="11.25" customHeight="1">
       <c r="A10" s="9" t="s">
         <v>17</v>
       </c>
@@ -779,7 +837,9 @@
       <c r="D10" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="13"/>
+      <c r="E10" s="13">
+        <v>59863</v>
+      </c>
       <c r="F10" s="13" t="s">
         <v>20</v>
       </c>
@@ -805,7 +865,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="10.9" customHeight="1">
+    <row r="11" ht="11.25" customHeight="1">
       <c r="A11" s="9" t="s">
         <v>17</v>
       </c>
@@ -818,7 +878,9 @@
       <c r="D11" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="13"/>
+      <c r="E11" s="13">
+        <v>59863</v>
+      </c>
       <c r="F11" s="13" t="s">
         <v>20</v>
       </c>
@@ -844,7 +906,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="10.9" customHeight="1">
+    <row r="12" ht="11.25" customHeight="1">
       <c r="A12" s="9" t="s">
         <v>17</v>
       </c>
@@ -857,7 +919,9 @@
       <c r="D12" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="13"/>
+      <c r="E12" s="13">
+        <v>59863</v>
+      </c>
       <c r="F12" s="13" t="s">
         <v>20</v>
       </c>
@@ -883,7 +947,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="10.9" customHeight="1">
+    <row r="13" ht="11.25" customHeight="1">
       <c r="A13" s="9" t="s">
         <v>17</v>
       </c>
@@ -896,7 +960,9 @@
       <c r="D13" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="13"/>
+      <c r="E13" s="13">
+        <v>59863</v>
+      </c>
       <c r="F13" s="13" t="s">
         <v>20</v>
       </c>
@@ -922,7 +988,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="10.9" customHeight="1">
+    <row r="14" ht="11.25" customHeight="1">
       <c r="A14" s="13" t="s">
         <v>23</v>
       </c>
@@ -935,7 +1001,9 @@
       <c r="D14" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E14" s="13"/>
+      <c r="E14" s="13">
+        <v>59863</v>
+      </c>
       <c r="F14" s="13" t="s">
         <v>20</v>
       </c>
@@ -961,7 +1029,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="10.9" customHeight="1">
+    <row r="15" ht="11.25" customHeight="1">
       <c r="A15" s="13" t="s">
         <v>23</v>
       </c>
@@ -974,7 +1042,9 @@
       <c r="D15" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E15" s="13"/>
+      <c r="E15" s="13">
+        <v>59863</v>
+      </c>
       <c r="F15" s="13" t="s">
         <v>20</v>
       </c>
@@ -1000,7 +1070,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="10.9" customHeight="1">
+    <row r="16" ht="11.25" customHeight="1">
       <c r="A16" s="13" t="s">
         <v>23</v>
       </c>
@@ -1013,7 +1083,9 @@
       <c r="D16" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E16" s="13"/>
+      <c r="E16" s="13">
+        <v>59863</v>
+      </c>
       <c r="F16" s="13" t="s">
         <v>20</v>
       </c>
@@ -1039,7 +1111,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="10.9" customHeight="1">
+    <row r="17" ht="11.25" customHeight="1">
       <c r="A17" s="13" t="s">
         <v>23</v>
       </c>
@@ -1052,7 +1124,9 @@
       <c r="D17" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E17" s="13"/>
+      <c r="E17" s="13">
+        <v>59863</v>
+      </c>
       <c r="F17" s="13" t="s">
         <v>20</v>
       </c>
@@ -1078,7 +1152,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="10.9" customHeight="1">
+    <row r="18" ht="11.25" customHeight="1">
       <c r="A18" s="13" t="s">
         <v>23</v>
       </c>
@@ -1091,7 +1165,9 @@
       <c r="D18" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E18" s="13"/>
+      <c r="E18" s="13">
+        <v>59863</v>
+      </c>
       <c r="F18" s="13" t="s">
         <v>20</v>
       </c>
@@ -1117,7 +1193,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="10.9" customHeight="1">
+    <row r="19" ht="11.25" customHeight="1">
       <c r="A19" s="13" t="s">
         <v>23</v>
       </c>
@@ -1130,7 +1206,9 @@
       <c r="D19" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E19" s="13"/>
+      <c r="E19" s="13">
+        <v>59863</v>
+      </c>
       <c r="F19" s="13" t="s">
         <v>20</v>
       </c>
@@ -1156,7 +1234,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="10.9" customHeight="1">
+    <row r="20" ht="11.25" customHeight="1">
       <c r="A20" s="13" t="s">
         <v>23</v>
       </c>
@@ -1169,7 +1247,9 @@
       <c r="D20" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E20" s="13"/>
+      <c r="E20" s="13">
+        <v>59863</v>
+      </c>
       <c r="F20" s="13" t="s">
         <v>20</v>
       </c>
@@ -1195,7 +1275,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="10.9" customHeight="1">
+    <row r="21" ht="11.25" customHeight="1">
       <c r="A21" s="13" t="s">
         <v>24</v>
       </c>
@@ -1208,7 +1288,9 @@
       <c r="D21" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E21" s="13"/>
+      <c r="E21" s="13">
+        <v>59863</v>
+      </c>
       <c r="F21" s="13" t="s">
         <v>20</v>
       </c>
@@ -1234,7 +1316,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="1:13" ht="10.9" customHeight="1">
+    <row r="22" ht="11.25" customHeight="1">
       <c r="A22" s="13" t="s">
         <v>24</v>
       </c>
@@ -1247,7 +1329,9 @@
       <c r="D22" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E22" s="13"/>
+      <c r="E22" s="13">
+        <v>59863</v>
+      </c>
       <c r="F22" s="13" t="s">
         <v>20</v>
       </c>
@@ -1273,7 +1357,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="10.9" customHeight="1">
+    <row r="23" ht="11.25" customHeight="1">
       <c r="A23" s="13" t="s">
         <v>24</v>
       </c>
@@ -1286,7 +1370,9 @@
       <c r="D23" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E23" s="13"/>
+      <c r="E23" s="13">
+        <v>59863</v>
+      </c>
       <c r="F23" s="13"/>
       <c r="G23" s="9" t="s">
         <v>21</v>
@@ -1310,7 +1396,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="10.9" customHeight="1">
+    <row r="24" ht="11.25" customHeight="1">
       <c r="A24" s="13" t="s">
         <v>24</v>
       </c>
@@ -1323,7 +1409,9 @@
       <c r="D24" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E24" s="13"/>
+      <c r="E24" s="13">
+        <v>59863</v>
+      </c>
       <c r="F24" s="13" t="s">
         <v>20</v>
       </c>
@@ -1349,7 +1437,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="1:13" ht="10.9" customHeight="1">
+    <row r="25" ht="11.25" customHeight="1">
       <c r="A25" s="13" t="s">
         <v>24</v>
       </c>
@@ -1362,7 +1450,9 @@
       <c r="D25" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E25" s="13"/>
+      <c r="E25" s="13">
+        <v>59863</v>
+      </c>
       <c r="F25" s="13" t="s">
         <v>20</v>
       </c>
@@ -1388,7 +1478,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="26" spans="1:13" ht="10.9" customHeight="1">
+    <row r="26" ht="11.25" customHeight="1">
       <c r="A26" s="13" t="s">
         <v>25</v>
       </c>
@@ -1401,7 +1491,9 @@
       <c r="D26" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E26" s="13"/>
+      <c r="E26" s="13">
+        <v>59863</v>
+      </c>
       <c r="F26" s="13" t="s">
         <v>20</v>
       </c>
@@ -1427,7 +1519,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="10.9" customHeight="1">
+    <row r="27" ht="11.25" customHeight="1">
       <c r="A27" s="13" t="s">
         <v>25</v>
       </c>
@@ -1440,7 +1532,9 @@
       <c r="D27" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E27" s="13"/>
+      <c r="E27" s="13">
+        <v>59863</v>
+      </c>
       <c r="F27" s="13" t="s">
         <v>20</v>
       </c>
@@ -1466,7 +1560,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="28" spans="1:13" ht="10.9" customHeight="1">
+    <row r="28" ht="11.25" customHeight="1">
       <c r="A28" s="13" t="s">
         <v>25</v>
       </c>
@@ -1479,7 +1573,9 @@
       <c r="D28" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E28" s="13"/>
+      <c r="E28" s="13">
+        <v>59863</v>
+      </c>
       <c r="F28" s="13" t="s">
         <v>20</v>
       </c>
@@ -1505,7 +1601,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="29" spans="1:13" ht="10.9" customHeight="1">
+    <row r="29" ht="11.25" customHeight="1">
       <c r="A29" s="13" t="s">
         <v>25</v>
       </c>
@@ -1518,7 +1614,9 @@
       <c r="D29" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E29" s="13"/>
+      <c r="E29" s="13">
+        <v>59863</v>
+      </c>
       <c r="F29" s="13" t="s">
         <v>20</v>
       </c>
@@ -1544,7 +1642,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="1:13" ht="10.9" customHeight="1">
+    <row r="30" ht="11.25" customHeight="1">
       <c r="A30" s="13" t="s">
         <v>25</v>
       </c>
@@ -1557,7 +1655,9 @@
       <c r="D30" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E30" s="13"/>
+      <c r="E30" s="13">
+        <v>59863</v>
+      </c>
       <c r="F30" s="13" t="s">
         <v>20</v>
       </c>
@@ -1583,7 +1683,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="31" spans="1:13" ht="10.9" customHeight="1">
+    <row r="31" ht="11.25" customHeight="1">
       <c r="A31" s="13" t="s">
         <v>25</v>
       </c>
@@ -1596,7 +1696,9 @@
       <c r="D31" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E31" s="13"/>
+      <c r="E31" s="13">
+        <v>59863</v>
+      </c>
       <c r="F31" s="13" t="s">
         <v>20</v>
       </c>
@@ -1622,7 +1724,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="32" spans="1:13" ht="10.9" customHeight="1">
+    <row r="32" ht="11.25" customHeight="1">
       <c r="A32" s="13" t="s">
         <v>25</v>
       </c>
@@ -1635,7 +1737,9 @@
       <c r="D32" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E32" s="13"/>
+      <c r="E32" s="13">
+        <v>59863</v>
+      </c>
       <c r="F32" s="13" t="s">
         <v>20</v>
       </c>
@@ -1661,7 +1765,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="33" spans="1:13" ht="10.9" customHeight="1">
+    <row r="33" ht="11.25" customHeight="1">
       <c r="A33" s="13" t="s">
         <v>25</v>
       </c>
@@ -1674,7 +1778,9 @@
       <c r="D33" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E33" s="13"/>
+      <c r="E33" s="13">
+        <v>59863</v>
+      </c>
       <c r="F33" s="13" t="s">
         <v>20</v>
       </c>
@@ -1700,7 +1806,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="1:13" ht="10.9" customHeight="1">
+    <row r="34" ht="11.25" customHeight="1">
       <c r="A34" s="13" t="s">
         <v>26</v>
       </c>
@@ -1713,7 +1819,9 @@
       <c r="D34" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E34" s="13"/>
+      <c r="E34" s="13">
+        <v>59863</v>
+      </c>
       <c r="F34" s="13" t="s">
         <v>20</v>
       </c>
@@ -1739,7 +1847,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="35" spans="1:13" ht="10.9" customHeight="1">
+    <row r="35" ht="11.25" customHeight="1">
       <c r="A35" s="13" t="s">
         <v>26</v>
       </c>
@@ -1752,7 +1860,9 @@
       <c r="D35" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E35" s="13"/>
+      <c r="E35" s="13">
+        <v>59863</v>
+      </c>
       <c r="F35" s="13" t="s">
         <v>20</v>
       </c>
@@ -1778,7 +1888,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="36" spans="1:13" ht="10.9" customHeight="1">
+    <row r="36" ht="11.25" customHeight="1">
       <c r="A36" s="13" t="s">
         <v>26</v>
       </c>
@@ -1791,7 +1901,9 @@
       <c r="D36" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E36" s="13"/>
+      <c r="E36" s="13">
+        <v>59863</v>
+      </c>
       <c r="F36" s="13" t="s">
         <v>20</v>
       </c>
@@ -1817,7 +1929,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="37" spans="1:13" ht="10.9" customHeight="1">
+    <row r="37" ht="11.25" customHeight="1">
       <c r="A37" s="13" t="s">
         <v>26</v>
       </c>
@@ -1830,7 +1942,9 @@
       <c r="D37" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E37" s="13"/>
+      <c r="E37" s="13">
+        <v>59863</v>
+      </c>
       <c r="F37" s="13" t="s">
         <v>20</v>
       </c>
@@ -1856,7 +1970,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="38" spans="1:13" ht="10.9" customHeight="1">
+    <row r="38" ht="11.25" customHeight="1">
       <c r="A38" s="13" t="s">
         <v>26</v>
       </c>
@@ -1869,7 +1983,9 @@
       <c r="D38" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E38" s="13"/>
+      <c r="E38" s="13">
+        <v>59863</v>
+      </c>
       <c r="F38" s="13" t="s">
         <v>20</v>
       </c>
@@ -1895,7 +2011,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="39" spans="1:13" ht="10.9" customHeight="1">
+    <row r="39" ht="11.25" customHeight="1">
       <c r="A39" s="13" t="s">
         <v>26</v>
       </c>
@@ -1908,7 +2024,9 @@
       <c r="D39" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E39" s="13"/>
+      <c r="E39" s="13">
+        <v>59863</v>
+      </c>
       <c r="F39" s="13" t="s">
         <v>20</v>
       </c>
@@ -1934,7 +2052,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="40" spans="1:13" ht="10.9" customHeight="1">
+    <row r="40" ht="11.25" customHeight="1">
       <c r="A40" s="13" t="s">
         <v>27</v>
       </c>
@@ -1947,7 +2065,9 @@
       <c r="D40" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E40" s="13"/>
+      <c r="E40" s="13">
+        <v>59863</v>
+      </c>
       <c r="F40" s="13" t="s">
         <v>20</v>
       </c>
@@ -1973,7 +2093,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="41" spans="1:13" ht="10.9" customHeight="1">
+    <row r="41" ht="11.25" customHeight="1">
       <c r="A41" s="13" t="s">
         <v>27</v>
       </c>
@@ -1986,7 +2106,9 @@
       <c r="D41" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E41" s="13"/>
+      <c r="E41" s="13">
+        <v>59863</v>
+      </c>
       <c r="F41" s="13" t="s">
         <v>20</v>
       </c>
@@ -2012,7 +2134,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="42" spans="1:13" ht="21.4" customHeight="1">
+    <row r="42" ht="21.75" customHeight="1">
       <c r="A42" s="13" t="s">
         <v>27</v>
       </c>
@@ -2025,7 +2147,9 @@
       <c r="D42" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E42" s="13"/>
+      <c r="E42" s="13">
+        <v>59863</v>
+      </c>
       <c r="F42" s="13" t="s">
         <v>20</v>
       </c>
@@ -2051,7 +2175,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="43" spans="1:13" ht="10.9" customHeight="1">
+    <row r="43" ht="11.25" customHeight="1">
       <c r="A43" s="13" t="s">
         <v>27</v>
       </c>
@@ -2064,7 +2188,9 @@
       <c r="D43" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E43" s="13"/>
+      <c r="E43" s="13">
+        <v>59863</v>
+      </c>
       <c r="F43" s="13" t="s">
         <v>20</v>
       </c>
@@ -2090,7 +2216,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="44" spans="1:13" ht="10.9" customHeight="1">
+    <row r="44" ht="11.25" customHeight="1">
       <c r="A44" s="13" t="s">
         <v>27</v>
       </c>
@@ -2103,7 +2229,9 @@
       <c r="D44" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E44" s="13"/>
+      <c r="E44" s="13">
+        <v>59863</v>
+      </c>
       <c r="F44" s="13" t="s">
         <v>20</v>
       </c>
@@ -2129,7 +2257,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="45" spans="1:13" ht="10.9" customHeight="1">
+    <row r="45" ht="11.25" customHeight="1">
       <c r="A45" s="13" t="s">
         <v>28</v>
       </c>
@@ -2142,7 +2270,9 @@
       <c r="D45" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E45" s="13"/>
+      <c r="E45" s="13">
+        <v>59863</v>
+      </c>
       <c r="F45" s="13" t="s">
         <v>20</v>
       </c>
@@ -2168,7 +2298,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="46" spans="1:13" ht="10.9" customHeight="1">
+    <row r="46" ht="11.25" customHeight="1">
       <c r="A46" s="16" t="s">
         <v>29</v>
       </c>
@@ -2189,10 +2319,12 @@
       <c r="M46" s="16"/>
     </row>
   </sheetData>
+  <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <pageSetup paperSize="9" pageOrder="downThenOver" orientation="portrait"/>
   <headerFooter>
-    <oddHeader>&amp;L&amp;"Aptos"&amp;10&amp;K000000 Interno General&amp;1#_x000D_</oddHeader>
+    <oddHeader>&amp;L&amp;"Aptos"&amp;10&amp;K000000 Interno General&amp;1#_x000D_&amp;C&amp;R</oddHeader>
   </headerFooter>
+  <extLst/>
 </worksheet>
 </file>
</xml_diff>